<commit_message>
Computed Position + table sort + Absolute floor label + detail redesign
- Position is now computed (Issuer-{|floor|%}-{maturity ddMMMyy}), not stored or
  imported; dedupedPosition() adds -1/-2 on collisions; form drops Position field
  (Issuer required); parser ignores xls Position, recomputes
- table: every column sortable, sort remembered (PortfolioStore, persisted),
  defaults to Next Reset ascending
- 0% floor labeled 'Absolute' (vs Hard) in app, image, and xlsx export
- drill-down redesigned: highlighted key-figures banner + reflowing section cards
- generator/example/template/image + README synced; 58 tests, core 100%/data 98%

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/assets/example-portfolio.xlsx
+++ b/app/assets/example-portfolio.xlsx
@@ -597,7 +597,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Aspida 12.25%-14Nov28</t>
+          <t>Aspida-0%-14Nov28</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -617,7 +617,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Absolute</t>
         </is>
       </c>
       <c r="H4" s="3" t="n">
@@ -677,7 +677,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Axa 65%-18Aug27</t>
+          <t>AXA-15%-18Aug27</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
@@ -757,7 +757,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Citi 15%-4Feb30 IRA</t>
+          <t>Citi-15%-04Feb30</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -839,7 +839,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>HSBC 92.25%-20Oct30</t>
+          <t>HSBC-15%-20Oct30</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
@@ -921,7 +921,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BNP 30%-6Jan31</t>
+          <t>BNP-30%-06Jan31</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -1003,7 +1003,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>NatBank 13.25%-16Apr29</t>
+          <t>Nat. Bank of Canada-30%-16Apr29</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
@@ -1083,7 +1083,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Axa 100%-20May32</t>
+          <t>AXA-20%-20May32</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -1163,7 +1163,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Citi 15%-1Dec29 ROTH</t>
+          <t>Citi-15%-01Dec29</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">

</xml_diff>

<commit_message>
Drop Position column from image + xlsx export (Issuer-led)
Image, xlsx export, generated example/template, and README summary now use the
app's column order (Issuer first, no Position). Position remains a computed
display name in the app (detail/edit/dedup); the parser still imports files that
do have a Position column (e.g. the real tracker). 58 tests, core 100%/data 98%.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/assets/example-portfolio.xlsx
+++ b/app/assets/example-portfolio.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V12"/>
+  <dimension ref="A1:U12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -465,7 +465,6 @@
     <col width="15" customWidth="1" min="19" max="19"/>
     <col width="15" customWidth="1" min="20" max="20"/>
     <col width="15" customWidth="1" min="21" max="21"/>
-    <col width="15" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -485,7 +484,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Position</t>
+          <t>Issuer</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -500,104 +499,99 @@
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
+          <t>Index</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
           <t>CAP</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>Part.</t>
         </is>
       </c>
-      <c r="F3" s="1" t="inlineStr">
+      <c r="G3" s="1" t="inlineStr">
         <is>
           <t>Floor</t>
         </is>
       </c>
-      <c r="G3" s="1" t="inlineStr">
+      <c r="H3" s="1" t="inlineStr">
         <is>
           <t>Floor Type</t>
         </is>
       </c>
-      <c r="H3" s="1" t="inlineStr">
+      <c r="I3" s="1" t="inlineStr">
         <is>
           <t>Strike</t>
         </is>
       </c>
-      <c r="I3" s="1" t="inlineStr">
+      <c r="J3" s="1" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="J3" s="1" t="inlineStr">
+      <c r="K3" s="1" t="inlineStr">
         <is>
           <t>Last Reset</t>
         </is>
       </c>
-      <c r="K3" s="1" t="inlineStr">
+      <c r="L3" s="1" t="inlineStr">
         <is>
           <t>Maturity</t>
         </is>
       </c>
-      <c r="L3" s="1" t="inlineStr">
+      <c r="M3" s="1" t="inlineStr">
         <is>
           <t>Days to Maturity</t>
         </is>
       </c>
-      <c r="M3" s="1" t="inlineStr">
+      <c r="N3" s="1" t="inlineStr">
         <is>
           <t>Reset Freq</t>
         </is>
       </c>
-      <c r="N3" s="1" t="inlineStr">
+      <c r="O3" s="1" t="inlineStr">
         <is>
           <t>Next Reset</t>
         </is>
       </c>
-      <c r="O3" s="1" t="inlineStr">
+      <c r="P3" s="1" t="inlineStr">
         <is>
           <t>Days to Reset</t>
         </is>
       </c>
-      <c r="P3" s="1" t="inlineStr">
+      <c r="Q3" s="1" t="inlineStr">
         <is>
           <t>Initial ($000)</t>
         </is>
       </c>
-      <c r="Q3" s="1" t="inlineStr">
+      <c r="R3" s="1" t="inlineStr">
         <is>
           <t>Realized ($000)</t>
         </is>
       </c>
-      <c r="R3" s="1" t="inlineStr">
+      <c r="S3" s="1" t="inlineStr">
         <is>
           <t>Proj Value @ Reset ($000)</t>
         </is>
       </c>
-      <c r="S3" s="1" t="inlineStr">
+      <c r="T3" s="1" t="inlineStr">
         <is>
           <t>Proj $ Gain @ Reset ($000)</t>
         </is>
       </c>
-      <c r="T3" s="1" t="inlineStr">
+      <c r="U3" s="1" t="inlineStr">
         <is>
           <t>Type</t>
-        </is>
-      </c>
-      <c r="U3" s="1" t="inlineStr">
-        <is>
-          <t>Issuer</t>
-        </is>
-      </c>
-      <c r="V3" s="1" t="inlineStr">
-        <is>
-          <t>Index</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Aspida-0%-14Nov28</t>
+          <t>Aspida</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -606,78 +600,73 @@
       <c r="C4" s="2" t="n">
         <v>0.1225</v>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
         <v>0.1225</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="F4" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="G4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Absolute</t>
         </is>
       </c>
-      <c r="H4" s="3" t="n">
+      <c r="I4" s="3" t="n">
         <v>6271.19</v>
       </c>
-      <c r="I4" s="4" t="n">
+      <c r="J4" s="4" t="n">
         <v>45247</v>
       </c>
-      <c r="J4" s="4" t="n">
+      <c r="K4" s="4" t="n">
         <v>45974</v>
       </c>
-      <c r="K4" s="4" t="n">
+      <c r="L4" s="4" t="n">
         <v>47071</v>
       </c>
-      <c r="L4" t="n">
+      <c r="M4" t="n">
         <v>884</v>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Annual</t>
         </is>
       </c>
-      <c r="N4" s="4" t="n">
+      <c r="O4" s="4" t="n">
         <v>46339</v>
       </c>
-      <c r="O4" t="n">
+      <c r="P4" t="n">
         <v>152</v>
       </c>
-      <c r="P4" s="5" t="n">
+      <c r="Q4" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="Q4" s="5" t="n">
+      <c r="R4" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="R4" s="5" t="n">
+      <c r="S4" s="5" t="n">
         <v>112.25</v>
       </c>
-      <c r="S4" s="5" t="n">
+      <c r="T4" s="5" t="n">
         <v>12.25</v>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>Non-Qual</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>Aspida</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>SPX</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AXA-15%-18Aug27</t>
+          <t>AXA</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
@@ -686,78 +675,73 @@
       <c r="C5" s="2" t="n">
         <v>-0.07000000000000001</v>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
         <v>0.65</v>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="F5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="G5" s="2" t="n">
         <v>-0.15</v>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
       </c>
-      <c r="H5" s="3" t="n">
+      <c r="I5" s="3" t="n">
         <v>9487.18</v>
-      </c>
-      <c r="I5" s="4" t="n">
-        <v>44426</v>
       </c>
       <c r="J5" s="4" t="n">
         <v>44426</v>
       </c>
       <c r="K5" s="4" t="n">
+        <v>44426</v>
+      </c>
+      <c r="L5" s="4" t="n">
         <v>46617</v>
       </c>
-      <c r="L5" t="n">
+      <c r="M5" t="n">
         <v>430</v>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>6-Year</t>
         </is>
       </c>
-      <c r="N5" s="4" t="n">
+      <c r="O5" s="4" t="n">
         <v>46617</v>
       </c>
-      <c r="O5" t="n">
+      <c r="P5" t="n">
         <v>430</v>
       </c>
-      <c r="P5" s="5" t="n">
+      <c r="Q5" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="Q5" s="5" t="n">
+      <c r="R5" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="R5" s="5" t="n">
+      <c r="S5" s="5" t="n">
         <v>93</v>
       </c>
-      <c r="S5" s="5" t="n">
+      <c r="T5" s="5" t="n">
         <v>-7.000000000000001</v>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>Non-Qual</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>AXA</t>
-        </is>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>SPX</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Citi-15%-04Feb30</t>
+          <t>Citi</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -768,78 +752,73 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
           <t>Uncapped</t>
         </is>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="F6" s="2" t="n">
         <v>1.02</v>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="G6" s="2" t="n">
         <v>-0.15</v>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
       </c>
-      <c r="H6" s="3" t="n">
+      <c r="I6" s="3" t="n">
         <v>5692.31</v>
-      </c>
-      <c r="I6" s="4" t="n">
-        <v>46022</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>46022</v>
       </c>
       <c r="K6" s="4" t="n">
+        <v>46022</v>
+      </c>
+      <c r="L6" s="4" t="n">
         <v>47518</v>
       </c>
-      <c r="L6" t="n">
+      <c r="M6" t="n">
         <v>1331</v>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>5-Year</t>
         </is>
       </c>
-      <c r="N6" s="4" t="n">
+      <c r="O6" s="4" t="n">
         <v>47518</v>
       </c>
-      <c r="O6" t="n">
+      <c r="P6" t="n">
         <v>1331</v>
       </c>
-      <c r="P6" s="5" t="n">
+      <c r="Q6" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="Q6" s="5" t="n">
+      <c r="R6" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="R6" s="5" t="n">
+      <c r="S6" s="5" t="n">
         <v>130.6</v>
       </c>
-      <c r="S6" s="5" t="n">
+      <c r="T6" s="5" t="n">
         <v>30.6</v>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>IRA</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>Citi</t>
-        </is>
-      </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>SPX</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>HSBC-15%-20Oct30</t>
+          <t>HSBC</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
@@ -850,78 +829,73 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
           <t>Uncapped</t>
         </is>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="F7" s="2" t="n">
         <v>0.9225</v>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="G7" s="2" t="n">
         <v>-0.15</v>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
       </c>
-      <c r="H7" s="3" t="n">
+      <c r="I7" s="3" t="n">
         <v>21142.86</v>
       </c>
-      <c r="I7" s="4" t="n">
+      <c r="J7" s="4" t="n">
         <v>45938</v>
       </c>
-      <c r="J7" s="4" t="n">
+      <c r="K7" s="4" t="n">
         <v>45933</v>
       </c>
-      <c r="K7" s="4" t="n">
+      <c r="L7" s="4" t="n">
         <v>47776</v>
       </c>
-      <c r="L7" t="n">
+      <c r="M7" t="n">
         <v>1589</v>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>5-Year</t>
         </is>
       </c>
-      <c r="N7" s="4" t="n">
+      <c r="O7" s="4" t="n">
         <v>47776</v>
       </c>
-      <c r="O7" t="n">
+      <c r="P7" t="n">
         <v>1589</v>
       </c>
-      <c r="P7" s="5" t="n">
+      <c r="Q7" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="Q7" s="5" t="n">
+      <c r="R7" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="R7" s="5" t="n">
+      <c r="S7" s="5" t="n">
         <v>136.9</v>
       </c>
-      <c r="S7" s="5" t="n">
+      <c r="T7" s="5" t="n">
         <v>36.9</v>
       </c>
-      <c r="T7" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>IRA</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>HSBC</t>
-        </is>
-      </c>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>NDX</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BNP-30%-06Jan31</t>
+          <t>BNP</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -932,78 +906,73 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
           <t>Uncapped</t>
         </is>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="F8" s="2" t="n">
         <v>1.05</v>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="G8" s="2" t="n">
         <v>-0.3</v>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>Soft</t>
         </is>
       </c>
-      <c r="H8" s="3" t="n">
+      <c r="I8" s="3" t="n">
         <v>11384.62</v>
-      </c>
-      <c r="I8" s="4" t="n">
-        <v>46022</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>46022</v>
       </c>
       <c r="K8" s="4" t="n">
+        <v>46022</v>
+      </c>
+      <c r="L8" s="4" t="n">
         <v>47854</v>
       </c>
-      <c r="L8" t="n">
+      <c r="M8" t="n">
         <v>1667</v>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>5-Year</t>
         </is>
       </c>
-      <c r="N8" s="4" t="n">
+      <c r="O8" s="4" t="n">
         <v>47854</v>
       </c>
-      <c r="O8" t="n">
+      <c r="P8" t="n">
         <v>1667</v>
       </c>
-      <c r="P8" s="5" t="n">
+      <c r="Q8" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="Q8" s="5" t="n">
+      <c r="R8" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="R8" s="5" t="n">
+      <c r="S8" s="5" t="n">
         <v>65</v>
       </c>
-      <c r="S8" s="5" t="n">
+      <c r="T8" s="5" t="n">
         <v>-35</v>
       </c>
-      <c r="T8" t="inlineStr">
+      <c r="U8" t="inlineStr">
         <is>
           <t>ROTH</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>BNP</t>
-        </is>
-      </c>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>SPX</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Nat. Bank of Canada-30%-16Apr29</t>
+          <t>Nat. Bank of Canada</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
@@ -1012,78 +981,73 @@
       <c r="C9" s="2" t="n">
         <v>0.0112</v>
       </c>
-      <c r="D9" s="2" t="n">
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>worst-of SPX/NDX/RUT</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
         <v>0.1325</v>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="F9" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="G9" s="2" t="n">
         <v>-0.3</v>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>Soft</t>
         </is>
       </c>
-      <c r="H9" s="3" t="n">
+      <c r="I9" s="3" t="n">
         <v>6583</v>
       </c>
-      <c r="I9" s="4" t="n">
+      <c r="J9" s="4" t="n">
         <v>46128</v>
       </c>
-      <c r="J9" s="4" t="n">
+      <c r="K9" s="4" t="n">
         <v>46158</v>
       </c>
-      <c r="K9" s="4" t="n">
+      <c r="L9" s="4" t="n">
         <v>47224</v>
       </c>
-      <c r="L9" t="n">
+      <c r="M9" t="n">
         <v>1037</v>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>Monthly</t>
         </is>
       </c>
-      <c r="N9" s="4" t="n">
+      <c r="O9" s="4" t="n">
         <v>46189</v>
       </c>
-      <c r="O9" t="n">
+      <c r="P9" t="n">
         <v>2</v>
       </c>
-      <c r="P9" s="5" t="n">
+      <c r="Q9" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="Q9" s="5" t="n">
+      <c r="R9" s="5" t="n">
         <v>1.1</v>
       </c>
-      <c r="R9" s="5" t="n">
+      <c r="S9" s="5" t="n">
         <v>102.22</v>
       </c>
-      <c r="S9" s="5" t="n">
+      <c r="T9" s="5" t="n">
         <v>1.12</v>
       </c>
-      <c r="T9" t="inlineStr">
+      <c r="U9" t="inlineStr">
         <is>
           <t>Non-Qual</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>Nat. Bank of Canada</t>
-        </is>
-      </c>
-      <c r="V9" t="inlineStr">
-        <is>
-          <t>worst-of SPX/NDX/RUT</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AXA-20%-20May32</t>
+          <t>AXA</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -1092,78 +1056,73 @@
       <c r="C10" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="2" t="n">
-        <v>1</v>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
       </c>
       <c r="E10" s="2" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="2" t="n">
         <v>-0.2</v>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
       </c>
-      <c r="H10" s="3" t="n">
+      <c r="I10" s="3" t="n">
         <v>34823.53</v>
-      </c>
-      <c r="I10" s="4" t="n">
-        <v>46162</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>46162</v>
       </c>
       <c r="K10" s="4" t="n">
+        <v>46162</v>
+      </c>
+      <c r="L10" s="4" t="n">
         <v>48354</v>
       </c>
-      <c r="L10" t="n">
+      <c r="M10" t="n">
         <v>2167</v>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>6-Year</t>
         </is>
       </c>
-      <c r="N10" s="4" t="n">
+      <c r="O10" s="4" t="n">
         <v>48354</v>
       </c>
-      <c r="O10" t="n">
+      <c r="P10" t="n">
         <v>2167</v>
       </c>
-      <c r="P10" s="5" t="n">
+      <c r="Q10" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="Q10" s="5" t="n">
+      <c r="R10" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="R10" s="5" t="n">
+      <c r="S10" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="S10" s="5" t="n">
+      <c r="T10" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="T10" t="inlineStr">
+      <c r="U10" t="inlineStr">
         <is>
           <t>IRA</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>AXA</t>
-        </is>
-      </c>
-      <c r="V10" t="inlineStr">
-        <is>
-          <t>NDX</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Citi-15%-01Dec29</t>
+          <t>Citi</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
@@ -1174,71 +1133,66 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
           <t>Uncapped</t>
         </is>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="F11" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="2" t="n">
+      <c r="G11" s="2" t="n">
         <v>-0.15</v>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
       </c>
-      <c r="H11" s="3" t="n">
+      <c r="I11" s="3" t="n">
         <v>6607.14</v>
-      </c>
-      <c r="I11" s="4" t="n">
-        <v>45989</v>
       </c>
       <c r="J11" s="4" t="n">
         <v>45989</v>
       </c>
       <c r="K11" s="4" t="n">
+        <v>45989</v>
+      </c>
+      <c r="L11" s="4" t="n">
         <v>47453</v>
       </c>
-      <c r="L11" t="n">
+      <c r="M11" t="n">
         <v>1266</v>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>4-Year</t>
         </is>
       </c>
-      <c r="N11" s="4" t="n">
+      <c r="O11" s="4" t="n">
         <v>47453</v>
       </c>
-      <c r="O11" t="n">
+      <c r="P11" t="n">
         <v>1266</v>
       </c>
-      <c r="P11" s="5" t="n">
+      <c r="Q11" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="Q11" s="5" t="n">
+      <c r="R11" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="R11" s="5" t="n">
+      <c r="S11" s="5" t="n">
         <v>112</v>
       </c>
-      <c r="S11" s="5" t="n">
+      <c r="T11" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="T11" t="inlineStr">
+      <c r="U11" t="inlineStr">
         <is>
           <t>ROTH</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>Citi</t>
-        </is>
-      </c>
-      <c r="V11" t="inlineStr">
-        <is>
-          <t>SPX</t>
         </is>
       </c>
     </row>
@@ -1251,32 +1205,31 @@
       <c r="B12" s="7" t="n"/>
       <c r="C12" s="7" t="n"/>
       <c r="D12" s="6" t="n"/>
-      <c r="E12" s="7" t="n"/>
+      <c r="E12" s="6" t="n"/>
       <c r="F12" s="7" t="n"/>
-      <c r="G12" s="6" t="n"/>
-      <c r="H12" s="8" t="n"/>
-      <c r="I12" s="9" t="n"/>
+      <c r="G12" s="7" t="n"/>
+      <c r="H12" s="6" t="n"/>
+      <c r="I12" s="8" t="n"/>
       <c r="J12" s="9" t="n"/>
       <c r="K12" s="9" t="n"/>
-      <c r="L12" s="6" t="n"/>
+      <c r="L12" s="9" t="n"/>
       <c r="M12" s="6" t="n"/>
-      <c r="N12" s="9" t="n"/>
-      <c r="O12" s="6" t="n"/>
-      <c r="P12" s="10" t="n">
+      <c r="N12" s="6" t="n"/>
+      <c r="O12" s="9" t="n"/>
+      <c r="P12" s="6" t="n"/>
+      <c r="Q12" s="10" t="n">
         <v>800</v>
       </c>
-      <c r="Q12" s="10" t="n">
+      <c r="R12" s="10" t="n">
         <v>1.1</v>
       </c>
-      <c r="R12" s="10" t="n">
+      <c r="S12" s="10" t="n">
         <v>851.97</v>
       </c>
-      <c r="S12" s="10" t="n">
+      <c r="T12" s="10" t="n">
         <v>50.87</v>
       </c>
-      <c r="T12" s="6" t="n"/>
       <c r="U12" s="6" t="n"/>
-      <c r="V12" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Refine column order to v1.2 (identity → inputs → outcome → timing → terms)
Lifts Initial/Realized next to the outcome columns so 'what I put in →
what it's worth' reads left-to-right, and splits the monitored
reset/maturity countdowns (Timing) from the static contract terms.
Applied to screen, schema v1.2, and gen_overview.py; regenerated
example/template xlsx + overview.png; updated the order test and default
sort index. Import still name-mapped (v1.0/v1.1 files load). 67 tests.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/assets/example-portfolio.xlsx
+++ b/app/assets/example-portfolio.xlsx
@@ -69,13 +69,13 @@
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -512,87 +512,87 @@
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
+          <t>Initial ($000)</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>Realized ($000)</t>
+        </is>
+      </c>
+      <c r="H3" s="1" t="inlineStr">
+        <is>
           <t>Proj Value @ Reset ($000)</t>
         </is>
       </c>
-      <c r="G3" s="1" t="inlineStr">
+      <c r="I3" s="1" t="inlineStr">
         <is>
           <t>Proj $ Gain @ Reset ($000)</t>
         </is>
       </c>
-      <c r="H3" s="1" t="inlineStr">
+      <c r="J3" s="1" t="inlineStr">
         <is>
           <t>Proj Gain @ Reset</t>
         </is>
       </c>
-      <c r="I3" s="1" t="inlineStr">
+      <c r="K3" s="1" t="inlineStr">
         <is>
           <t>Index Gain %</t>
         </is>
       </c>
-      <c r="J3" s="1" t="inlineStr">
+      <c r="L3" s="1" t="inlineStr">
+        <is>
+          <t>Next Reset</t>
+        </is>
+      </c>
+      <c r="M3" s="1" t="inlineStr">
+        <is>
+          <t>Days to Reset</t>
+        </is>
+      </c>
+      <c r="N3" s="1" t="inlineStr">
+        <is>
+          <t>Maturity</t>
+        </is>
+      </c>
+      <c r="O3" s="1" t="inlineStr">
+        <is>
+          <t>Days to Maturity</t>
+        </is>
+      </c>
+      <c r="P3" s="1" t="inlineStr">
         <is>
           <t>CAP</t>
         </is>
       </c>
-      <c r="K3" s="1" t="inlineStr">
+      <c r="Q3" s="1" t="inlineStr">
         <is>
           <t>Part.</t>
         </is>
       </c>
-      <c r="L3" s="1" t="inlineStr">
+      <c r="R3" s="1" t="inlineStr">
         <is>
           <t>Floor</t>
         </is>
       </c>
-      <c r="M3" s="1" t="inlineStr">
+      <c r="S3" s="1" t="inlineStr">
         <is>
           <t>Strike</t>
         </is>
       </c>
-      <c r="N3" s="1" t="inlineStr">
-        <is>
-          <t>Next Reset</t>
-        </is>
-      </c>
-      <c r="O3" s="1" t="inlineStr">
-        <is>
-          <t>Days to Reset</t>
-        </is>
-      </c>
-      <c r="P3" s="1" t="inlineStr">
-        <is>
-          <t>Maturity</t>
-        </is>
-      </c>
-      <c r="Q3" s="1" t="inlineStr">
-        <is>
-          <t>Days to Maturity</t>
-        </is>
-      </c>
-      <c r="R3" s="1" t="inlineStr">
+      <c r="T3" s="1" t="inlineStr">
         <is>
           <t>Reset Freq</t>
         </is>
       </c>
-      <c r="S3" s="1" t="inlineStr">
+      <c r="U3" s="1" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="T3" s="1" t="inlineStr">
+      <c r="V3" s="1" t="inlineStr">
         <is>
           <t>Last Reset</t>
-        </is>
-      </c>
-      <c r="U3" s="1" t="inlineStr">
-        <is>
-          <t>Initial ($000)</t>
-        </is>
-      </c>
-      <c r="V3" s="1" t="inlineStr">
-        <is>
-          <t>Realized ($000)</t>
         </is>
       </c>
       <c r="W3" s="1" t="inlineStr">
@@ -633,60 +633,60 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="2" t="n">
         <v>112.25</v>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="I4" s="2" t="n">
         <v>12.25</v>
-      </c>
-      <c r="H4" s="3" t="n">
-        <v>0.1225</v>
-      </c>
-      <c r="I4" s="3" t="n">
-        <v>0.18</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>0.1225</v>
       </c>
       <c r="K4" s="3" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>46339</v>
+      </c>
+      <c r="M4" t="n">
+        <v>152</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>47071</v>
+      </c>
+      <c r="O4" t="n">
+        <v>884</v>
+      </c>
+      <c r="P4" s="3" t="n">
+        <v>0.1225</v>
+      </c>
+      <c r="Q4" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="L4" s="3" t="n">
+      <c r="R4" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="M4" s="4" t="n">
+      <c r="S4" s="5" t="n">
         <v>6271.19</v>
       </c>
-      <c r="N4" s="5" t="n">
-        <v>46339</v>
-      </c>
-      <c r="O4" t="n">
-        <v>152</v>
-      </c>
-      <c r="P4" s="5" t="n">
-        <v>47071</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>884</v>
-      </c>
-      <c r="R4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>Annual</t>
         </is>
       </c>
-      <c r="S4" s="5" t="n">
+      <c r="U4" s="4" t="n">
         <v>45247</v>
       </c>
-      <c r="T4" s="5" t="n">
+      <c r="V4" s="4" t="n">
         <v>45974</v>
       </c>
-      <c r="U4" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="V4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="W4" s="4" t="n"/>
-      <c r="X4" s="4" t="n"/>
+      <c r="W4" s="5" t="n"/>
+      <c r="X4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -715,60 +715,60 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="2" t="n">
         <v>93</v>
       </c>
-      <c r="G5" s="2" t="n">
+      <c r="I5" s="2" t="n">
         <v>-7.000000000000001</v>
       </c>
-      <c r="H5" s="3" t="n">
+      <c r="J5" s="3" t="n">
         <v>-0.07000000000000001</v>
       </c>
-      <c r="I5" s="3" t="n">
+      <c r="K5" s="3" t="n">
         <v>-0.22</v>
       </c>
-      <c r="J5" s="3" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="K5" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="L5" s="3" t="n">
-        <v>-0.15</v>
-      </c>
-      <c r="M5" s="4" t="n">
-        <v>9487.18</v>
-      </c>
-      <c r="N5" s="5" t="n">
+      <c r="L5" s="4" t="n">
+        <v>46617</v>
+      </c>
+      <c r="M5" t="n">
+        <v>430</v>
+      </c>
+      <c r="N5" s="4" t="n">
         <v>46617</v>
       </c>
       <c r="O5" t="n">
         <v>430</v>
       </c>
-      <c r="P5" s="5" t="n">
-        <v>46617</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>430</v>
-      </c>
-      <c r="R5" t="inlineStr">
+      <c r="P5" s="3" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="Q5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="R5" s="3" t="n">
+        <v>-0.15</v>
+      </c>
+      <c r="S5" s="5" t="n">
+        <v>9487.18</v>
+      </c>
+      <c r="T5" t="inlineStr">
         <is>
           <t>Inception</t>
         </is>
       </c>
-      <c r="S5" s="5" t="n">
+      <c r="U5" s="4" t="n">
         <v>44426</v>
       </c>
-      <c r="T5" s="5" t="n">
+      <c r="V5" s="4" t="n">
         <v>44426</v>
       </c>
-      <c r="U5" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="V5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="W5" s="4" t="n"/>
-      <c r="X5" s="4" t="n"/>
+      <c r="W5" s="5" t="n"/>
+      <c r="X5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -797,60 +797,60 @@
         </is>
       </c>
       <c r="F6" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="2" t="n">
         <v>130.6</v>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="I6" s="2" t="n">
         <v>30.6</v>
       </c>
-      <c r="H6" s="3" t="n">
+      <c r="J6" s="3" t="n">
         <v>0.306</v>
       </c>
-      <c r="I6" s="3" t="n">
+      <c r="K6" s="3" t="n">
         <v>0.3</v>
       </c>
-      <c r="J6" s="3" t="n">
-        <v>9.99</v>
-      </c>
-      <c r="K6" s="3" t="n">
-        <v>1.02</v>
-      </c>
-      <c r="L6" s="3" t="n">
-        <v>-0.15</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>5692.31</v>
-      </c>
-      <c r="N6" s="5" t="n">
+      <c r="L6" s="4" t="n">
+        <v>47518</v>
+      </c>
+      <c r="M6" t="n">
+        <v>1331</v>
+      </c>
+      <c r="N6" s="4" t="n">
         <v>47518</v>
       </c>
       <c r="O6" t="n">
         <v>1331</v>
       </c>
-      <c r="P6" s="5" t="n">
-        <v>47518</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>1331</v>
-      </c>
-      <c r="R6" t="inlineStr">
+      <c r="P6" s="3" t="n">
+        <v>9.99</v>
+      </c>
+      <c r="Q6" s="3" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="R6" s="3" t="n">
+        <v>-0.15</v>
+      </c>
+      <c r="S6" s="5" t="n">
+        <v>5692.31</v>
+      </c>
+      <c r="T6" t="inlineStr">
         <is>
           <t>Inception</t>
         </is>
       </c>
-      <c r="S6" s="5" t="n">
+      <c r="U6" s="4" t="n">
         <v>46022</v>
       </c>
-      <c r="T6" s="5" t="n">
+      <c r="V6" s="4" t="n">
         <v>46022</v>
       </c>
-      <c r="U6" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="V6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="W6" s="4" t="n"/>
-      <c r="X6" s="4" t="n"/>
+      <c r="W6" s="5" t="n"/>
+      <c r="X6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -879,60 +879,60 @@
         </is>
       </c>
       <c r="F7" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="2" t="n">
         <v>136.9</v>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="I7" s="2" t="n">
         <v>36.9</v>
       </c>
-      <c r="H7" s="3" t="n">
+      <c r="J7" s="3" t="n">
         <v>0.369</v>
       </c>
-      <c r="I7" s="3" t="n">
+      <c r="K7" s="3" t="n">
         <v>0.4</v>
       </c>
-      <c r="J7" s="3" t="n">
-        <v>9.99</v>
-      </c>
-      <c r="K7" s="3" t="n">
-        <v>0.9225</v>
-      </c>
-      <c r="L7" s="3" t="n">
-        <v>-0.15</v>
-      </c>
-      <c r="M7" s="4" t="n">
-        <v>21142.86</v>
-      </c>
-      <c r="N7" s="5" t="n">
+      <c r="L7" s="4" t="n">
+        <v>47776</v>
+      </c>
+      <c r="M7" t="n">
+        <v>1589</v>
+      </c>
+      <c r="N7" s="4" t="n">
         <v>47776</v>
       </c>
       <c r="O7" t="n">
         <v>1589</v>
       </c>
-      <c r="P7" s="5" t="n">
-        <v>47776</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>1589</v>
-      </c>
-      <c r="R7" t="inlineStr">
+      <c r="P7" s="3" t="n">
+        <v>9.99</v>
+      </c>
+      <c r="Q7" s="3" t="n">
+        <v>0.9225</v>
+      </c>
+      <c r="R7" s="3" t="n">
+        <v>-0.15</v>
+      </c>
+      <c r="S7" s="5" t="n">
+        <v>21142.86</v>
+      </c>
+      <c r="T7" t="inlineStr">
         <is>
           <t>Inception</t>
         </is>
       </c>
-      <c r="S7" s="5" t="n">
+      <c r="U7" s="4" t="n">
         <v>45938</v>
       </c>
-      <c r="T7" s="5" t="n">
+      <c r="V7" s="4" t="n">
         <v>45933</v>
       </c>
-      <c r="U7" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="V7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="W7" s="4" t="n"/>
-      <c r="X7" s="4" t="n"/>
+      <c r="W7" s="5" t="n"/>
+      <c r="X7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -961,60 +961,60 @@
         </is>
       </c>
       <c r="F8" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="2" t="n">
         <v>65</v>
       </c>
-      <c r="G8" s="2" t="n">
+      <c r="I8" s="2" t="n">
         <v>-35</v>
       </c>
-      <c r="H8" s="3" t="n">
+      <c r="J8" s="3" t="n">
         <v>-0.35</v>
       </c>
-      <c r="I8" s="3" t="n">
+      <c r="K8" s="3" t="n">
         <v>-0.35</v>
       </c>
-      <c r="J8" s="3" t="n">
-        <v>9.99</v>
-      </c>
-      <c r="K8" s="3" t="n">
-        <v>1.05</v>
-      </c>
-      <c r="L8" s="3" t="n">
-        <v>-0.3</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>11384.62</v>
-      </c>
-      <c r="N8" s="5" t="n">
+      <c r="L8" s="4" t="n">
+        <v>47854</v>
+      </c>
+      <c r="M8" t="n">
+        <v>1667</v>
+      </c>
+      <c r="N8" s="4" t="n">
         <v>47854</v>
       </c>
       <c r="O8" t="n">
         <v>1667</v>
       </c>
-      <c r="P8" s="5" t="n">
-        <v>47854</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>1667</v>
-      </c>
-      <c r="R8" t="inlineStr">
+      <c r="P8" s="3" t="n">
+        <v>9.99</v>
+      </c>
+      <c r="Q8" s="3" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="R8" s="3" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="S8" s="5" t="n">
+        <v>11384.62</v>
+      </c>
+      <c r="T8" t="inlineStr">
         <is>
           <t>Inception</t>
         </is>
       </c>
-      <c r="S8" s="5" t="n">
+      <c r="U8" s="4" t="n">
         <v>46022</v>
       </c>
-      <c r="T8" s="5" t="n">
+      <c r="V8" s="4" t="n">
         <v>46022</v>
       </c>
-      <c r="U8" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="V8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="W8" s="4" t="n"/>
-      <c r="X8" s="4" t="n"/>
+      <c r="W8" s="5" t="n"/>
+      <c r="X8" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1043,62 +1043,62 @@
         </is>
       </c>
       <c r="F9" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="H9" s="2" t="n">
         <v>102.22</v>
       </c>
-      <c r="G9" s="2" t="n">
+      <c r="I9" s="2" t="n">
         <v>1.12</v>
       </c>
-      <c r="H9" s="3" t="n">
+      <c r="J9" s="3" t="n">
         <v>0.0112</v>
       </c>
-      <c r="I9" s="3" t="n">
+      <c r="K9" s="3" t="n">
         <v>0.0847</v>
       </c>
-      <c r="J9" s="3" t="n">
+      <c r="L9" s="4" t="n">
+        <v>46189</v>
+      </c>
+      <c r="M9" t="n">
+        <v>2</v>
+      </c>
+      <c r="N9" s="4" t="n">
+        <v>47224</v>
+      </c>
+      <c r="O9" t="n">
+        <v>1037</v>
+      </c>
+      <c r="P9" s="3" t="n">
         <v>0.1325</v>
       </c>
-      <c r="K9" s="3" t="n">
+      <c r="Q9" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="L9" s="3" t="n">
+      <c r="R9" s="3" t="n">
         <v>-0.3</v>
       </c>
-      <c r="M9" s="4" t="n">
+      <c r="S9" s="5" t="n">
         <v>6583</v>
       </c>
-      <c r="N9" s="5" t="n">
-        <v>46189</v>
-      </c>
-      <c r="O9" t="n">
-        <v>2</v>
-      </c>
-      <c r="P9" s="5" t="n">
-        <v>47224</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>1037</v>
-      </c>
-      <c r="R9" t="inlineStr">
+      <c r="T9" t="inlineStr">
         <is>
           <t>Monthly</t>
         </is>
       </c>
-      <c r="S9" s="5" t="n">
+      <c r="U9" s="4" t="n">
         <v>46128</v>
       </c>
-      <c r="T9" s="5" t="n">
+      <c r="V9" s="4" t="n">
         <v>46158</v>
       </c>
-      <c r="U9" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="V9" s="2" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="W9" s="4" t="n">
+      <c r="W9" s="5" t="n">
         <v>27290</v>
       </c>
-      <c r="X9" s="4" t="n">
+      <c r="X9" s="5" t="n">
         <v>2719</v>
       </c>
     </row>
@@ -1134,55 +1134,55 @@
       <c r="G10" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="3" t="n">
+      <c r="H10" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="I10" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I10" s="3" t="n">
+      <c r="J10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="3" t="n">
         <v>-0.15</v>
       </c>
-      <c r="J10" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K10" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="L10" s="3" t="n">
-        <v>-0.2</v>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>34823.53</v>
-      </c>
-      <c r="N10" s="5" t="n">
+      <c r="L10" s="4" t="n">
+        <v>48354</v>
+      </c>
+      <c r="M10" t="n">
+        <v>2167</v>
+      </c>
+      <c r="N10" s="4" t="n">
         <v>48354</v>
       </c>
       <c r="O10" t="n">
         <v>2167</v>
       </c>
-      <c r="P10" s="5" t="n">
-        <v>48354</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>2167</v>
-      </c>
-      <c r="R10" t="inlineStr">
+      <c r="P10" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q10" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="R10" s="3" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="S10" s="5" t="n">
+        <v>34823.53</v>
+      </c>
+      <c r="T10" t="inlineStr">
         <is>
           <t>Inception</t>
         </is>
       </c>
-      <c r="S10" s="5" t="n">
+      <c r="U10" s="4" t="n">
         <v>46162</v>
       </c>
-      <c r="T10" s="5" t="n">
+      <c r="V10" s="4" t="n">
         <v>46162</v>
       </c>
-      <c r="U10" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="V10" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="W10" s="4" t="n"/>
-      <c r="X10" s="4" t="n"/>
+      <c r="W10" s="5" t="n"/>
+      <c r="X10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1211,60 +1211,60 @@
         </is>
       </c>
       <c r="F11" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="2" t="n">
         <v>112</v>
       </c>
-      <c r="G11" s="2" t="n">
+      <c r="I11" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="H11" s="3" t="n">
+      <c r="J11" s="3" t="n">
         <v>0.12</v>
       </c>
-      <c r="I11" s="3" t="n">
+      <c r="K11" s="3" t="n">
         <v>0.12</v>
       </c>
-      <c r="J11" s="3" t="n">
-        <v>9.99</v>
-      </c>
-      <c r="K11" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="L11" s="3" t="n">
-        <v>-0.15</v>
-      </c>
-      <c r="M11" s="4" t="n">
-        <v>6607.14</v>
-      </c>
-      <c r="N11" s="5" t="n">
+      <c r="L11" s="4" t="n">
+        <v>47453</v>
+      </c>
+      <c r="M11" t="n">
+        <v>1266</v>
+      </c>
+      <c r="N11" s="4" t="n">
         <v>47453</v>
       </c>
       <c r="O11" t="n">
         <v>1266</v>
       </c>
-      <c r="P11" s="5" t="n">
-        <v>47453</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>1266</v>
-      </c>
-      <c r="R11" t="inlineStr">
+      <c r="P11" s="3" t="n">
+        <v>9.99</v>
+      </c>
+      <c r="Q11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="R11" s="3" t="n">
+        <v>-0.15</v>
+      </c>
+      <c r="S11" s="5" t="n">
+        <v>6607.14</v>
+      </c>
+      <c r="T11" t="inlineStr">
         <is>
           <t>Inception</t>
         </is>
       </c>
-      <c r="S11" s="5" t="n">
+      <c r="U11" s="4" t="n">
         <v>45989</v>
       </c>
-      <c r="T11" s="5" t="n">
+      <c r="V11" s="4" t="n">
         <v>45989</v>
       </c>
-      <c r="U11" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="V11" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="W11" s="4" t="n"/>
-      <c r="X11" s="4" t="n"/>
+      <c r="W11" s="5" t="n"/>
+      <c r="X11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -1277,32 +1277,32 @@
       <c r="D12" s="6" t="n"/>
       <c r="E12" s="6" t="n"/>
       <c r="F12" s="7" t="n">
+        <v>800</v>
+      </c>
+      <c r="G12" s="7" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="H12" s="7" t="n">
         <v>851.97</v>
       </c>
-      <c r="G12" s="7" t="n">
+      <c r="I12" s="7" t="n">
         <v>50.87</v>
       </c>
-      <c r="H12" s="8" t="n"/>
-      <c r="I12" s="8" t="n"/>
       <c r="J12" s="8" t="n"/>
       <c r="K12" s="8" t="n"/>
-      <c r="L12" s="8" t="n"/>
-      <c r="M12" s="9" t="n"/>
-      <c r="N12" s="10" t="n"/>
+      <c r="L12" s="9" t="n"/>
+      <c r="M12" s="6" t="n"/>
+      <c r="N12" s="9" t="n"/>
       <c r="O12" s="6" t="n"/>
-      <c r="P12" s="10" t="n"/>
-      <c r="Q12" s="6" t="n"/>
-      <c r="R12" s="6" t="n"/>
+      <c r="P12" s="8" t="n"/>
+      <c r="Q12" s="8" t="n"/>
+      <c r="R12" s="8" t="n"/>
       <c r="S12" s="10" t="n"/>
-      <c r="T12" s="10" t="n"/>
-      <c r="U12" s="7" t="n">
-        <v>800</v>
-      </c>
-      <c r="V12" s="7" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="W12" s="9" t="n"/>
-      <c r="X12" s="9" t="n"/>
+      <c r="T12" s="6" t="n"/>
+      <c r="U12" s="9" t="n"/>
+      <c r="V12" s="9" t="n"/>
+      <c r="W12" s="10" t="n"/>
+      <c r="X12" s="10" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Reconcile projected value to the real tracker; clear-data backup warning
- projValue now reinvests realized into the base, matching the Zucker
  tracker formulas R=(P+Q)*(1+C), S=R-(P+Q): projValue=(initial+realized)*
  (1+gain), unrealized=(initial+realized)*gain. Verified against actual
  sheet rows (e.g. AIG (100+36.8)*1.105=151.16). Updated model, payoff,
  gen_overview + regenerated example/overview.png + tests.
- Clear all data: stronger 'cannot be undone' warning + an Export backup
  button in the typed-confirm dialog. 75 tests.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/assets/example-portfolio.xlsx
+++ b/app/assets/example-portfolio.xlsx
@@ -1049,10 +1049,10 @@
         <v>1.1</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>102.22</v>
+        <v>102.23232</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>1.12</v>
+        <v>1.13232</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>0.0112</v>
@@ -1283,10 +1283,10 @@
         <v>1.1</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>851.97</v>
+        <v>851.9823200000001</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>50.87</v>
+        <v>50.88231999999999</v>
       </c>
       <c r="J12" s="8" t="n"/>
       <c r="K12" s="8" t="n"/>

</xml_diff>

<commit_message>
example: add a max-loss Floor contract; document the 4th downside type
Regenerate the sample/template/overview from gen_overview.py with a 9th
contract (MAREX, ^RUT, −10% Floor) so the example exercises all four downside
types end-to-end (−18% move clamps to −10%, vs −8% for a buffer). Updates the
overview.png, README protection-type docs + example table, and the xlsx legend/
Instructions. Bumps count/total assertions (8→9, $800→$900, $851.98→$941.98)
and asserts the Floor type imports as FloorType.floor.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/assets/example-portfolio.xlsx
+++ b/app/assets/example-portfolio.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X12"/>
+  <dimension ref="A1:X13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -480,7 +480,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Floor Type: Protected (0% floor), Hard (buffer — absorbs first |floor|), Soft (barrier — full loss if breached) | CAP 9.99 = uncapped | $ columns in $000s</t>
+          <t>Floor Type: Protected (0% floor), Hard (buffer — absorbs first |floor|), Soft (barrier — full loss if breached), Floor (max loss — lose only down to the floor) | CAP 9.99 = uncapped | $ columns in $000s</t>
         </is>
       </c>
     </row>
@@ -1267,42 +1267,124 @@
       <c r="X11" s="5" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>MAREX-10%-12Jun31</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>MAREX</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Non-Qual</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>^RUT</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Floor</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>-10</v>
+      </c>
+      <c r="J12" s="3" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="K12" s="3" t="n">
+        <v>-0.18</v>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>48011</v>
+      </c>
+      <c r="M12" t="n">
+        <v>1824</v>
+      </c>
+      <c r="N12" s="4" t="n">
+        <v>48011</v>
+      </c>
+      <c r="O12" t="n">
+        <v>1824</v>
+      </c>
+      <c r="P12" s="3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q12" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="R12" s="3" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="S12" s="5" t="n">
+        <v>3597.56</v>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>Inception</t>
+        </is>
+      </c>
+      <c r="U12" s="4" t="n">
+        <v>46185</v>
+      </c>
+      <c r="V12" s="4" t="n">
+        <v>46185</v>
+      </c>
+      <c r="W12" s="5" t="n"/>
+      <c r="X12" s="5" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B12" s="6" t="n"/>
-      <c r="C12" s="6" t="n"/>
-      <c r="D12" s="6" t="n"/>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="7" t="n">
-        <v>800</v>
-      </c>
-      <c r="G12" s="7" t="n">
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="7" t="n">
+        <v>900</v>
+      </c>
+      <c r="G13" s="7" t="n">
         <v>1.1</v>
       </c>
-      <c r="H12" s="7" t="n">
-        <v>851.9823200000001</v>
-      </c>
-      <c r="I12" s="7" t="n">
-        <v>50.88231999999999</v>
-      </c>
-      <c r="J12" s="8" t="n"/>
-      <c r="K12" s="8" t="n"/>
-      <c r="L12" s="9" t="n"/>
-      <c r="M12" s="6" t="n"/>
-      <c r="N12" s="9" t="n"/>
-      <c r="O12" s="6" t="n"/>
-      <c r="P12" s="8" t="n"/>
-      <c r="Q12" s="8" t="n"/>
-      <c r="R12" s="8" t="n"/>
-      <c r="S12" s="10" t="n"/>
-      <c r="T12" s="6" t="n"/>
-      <c r="U12" s="9" t="n"/>
-      <c r="V12" s="9" t="n"/>
-      <c r="W12" s="10" t="n"/>
-      <c r="X12" s="10" t="n"/>
+      <c r="H13" s="7" t="n">
+        <v>941.9823200000001</v>
+      </c>
+      <c r="I13" s="7" t="n">
+        <v>40.88231999999999</v>
+      </c>
+      <c r="J13" s="8" t="n"/>
+      <c r="K13" s="8" t="n"/>
+      <c r="L13" s="9" t="n"/>
+      <c r="M13" s="6" t="n"/>
+      <c r="N13" s="9" t="n"/>
+      <c r="O13" s="6" t="n"/>
+      <c r="P13" s="8" t="n"/>
+      <c r="Q13" s="8" t="n"/>
+      <c r="R13" s="8" t="n"/>
+      <c r="S13" s="10" t="n"/>
+      <c r="T13" s="6" t="n"/>
+      <c r="U13" s="9" t="n"/>
+      <c r="V13" s="9" t="n"/>
+      <c r="W13" s="10" t="n"/>
+      <c r="X13" s="10" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Rename floor types: Floor / Hard-buffer / Soft-buffer
Per request, rename the downside-protection labels and fold the 0% case in:
- 'Protected' (0% floor) → 'Floor' (a Floor at 0%)
- 'Hard' (buffer) → 'Hard-buffer'
- 'Soft' (barrier) → 'Soft-buffer'

Labels are display-only (protectionType); the internal FloorType{hard,soft,floor}
enum is unchanged, so JSON-stored portfolios need no migration. The importer
still accepts legacy Protected/Hard/Soft tokens, so existing .xlsx files import
correctly. (Considered Floor→Hard but rejected it — legacy 'Hard' means buffer.)
Updates models/format/info page/hero, the importer + export legend/instructions,
gen_overview.py + regenerated example/template/overview.png, README, and tests.
Also aligns the example's income-note projection to cap/12.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/assets/example-portfolio.xlsx
+++ b/app/assets/example-portfolio.xlsx
@@ -480,7 +480,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Floor Type: Protected (0% floor), Hard (buffer — absorbs first |floor|), Soft (barrier — full loss if breached), Floor (max loss — lose only down to the floor) | CAP 9.99 = uncapped | $ columns in $000s</t>
+          <t>Floor Type: Floor (max loss — lose only down to the floor; 0% floor = no loss), Hard-buffer (absorbs first |floor|, lose beyond), Soft-buffer (barrier — full loss if breached) | CAP 9.99 = uncapped | $ columns in $000s</t>
         </is>
       </c>
     </row>
@@ -629,7 +629,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Protected</t>
+          <t>Floor</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
@@ -711,7 +711,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Hard-buffer</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
@@ -793,7 +793,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Hard-buffer</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
@@ -875,7 +875,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Hard-buffer</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
@@ -957,7 +957,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Soft</t>
+          <t>Soft-buffer</t>
         </is>
       </c>
       <c r="F8" s="2" t="n">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Soft</t>
+          <t>Soft-buffer</t>
         </is>
       </c>
       <c r="F9" s="2" t="n">
@@ -1049,13 +1049,13 @@
         <v>1.1</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>102.23232</v>
+        <v>102.2163125</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>1.13232</v>
+        <v>1.1163125</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>0.0112</v>
+        <v>0.01104166666666667</v>
       </c>
       <c r="K9" s="3" t="n">
         <v>0.0847</v>
@@ -1125,7 +1125,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Hard-buffer</t>
         </is>
       </c>
       <c r="F10" s="2" t="n">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Hard-buffer</t>
         </is>
       </c>
       <c r="F11" s="2" t="n">
@@ -1365,10 +1365,10 @@
         <v>1.1</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>941.9823200000001</v>
+        <v>941.9663125</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>40.88231999999999</v>
+        <v>40.86631249999999</v>
       </c>
       <c r="J13" s="8" t="n"/>
       <c r="K13" s="8" t="n"/>

</xml_diff>

<commit_message>
Shorten floor-type labels back to Hard / Soft (save screen space)
Floor types are now Floor / Hard / Soft (Hard=buffer, Soft=barrier, Floor=
max-loss incl. 0%). Hard/Soft match the legacy import tokens, so no collision
and no relabeling. Display-only label change (internal FloorType enum + JSON
unchanged). Updates UI/info/hero, export legend + instructions, gen_overview.py
+ regenerated example/template/overview.png, README, tests, memory.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/assets/example-portfolio.xlsx
+++ b/app/assets/example-portfolio.xlsx
@@ -480,7 +480,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Floor Type: Floor (max loss — lose only down to the floor; 0% floor = no loss), Hard-buffer (absorbs first |floor|, lose beyond), Soft-buffer (barrier — full loss if breached) | CAP 9.99 = uncapped | $ columns in $000s</t>
+          <t>Floor Type: Floor (max loss — lose only down to the floor; 0% floor = no loss), Hard (buffer — absorbs first |floor|, lose beyond), Soft (barrier — full loss if breached) | CAP 9.99 = uncapped | $ columns in $000s</t>
         </is>
       </c>
     </row>
@@ -711,7 +711,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Hard-buffer</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
@@ -793,7 +793,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Hard-buffer</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
@@ -875,7 +875,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Hard-buffer</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
@@ -957,7 +957,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Soft-buffer</t>
+          <t>Soft</t>
         </is>
       </c>
       <c r="F8" s="2" t="n">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Soft-buffer</t>
+          <t>Soft</t>
         </is>
       </c>
       <c r="F9" s="2" t="n">
@@ -1125,7 +1125,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Hard-buffer</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="F10" s="2" t="n">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Hard-buffer</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="F11" s="2" t="n">

</xml_diff>

<commit_message>
Docs: regenerate example assets for Start Date / Once + Inception column
Run gen_overview.py with the renamed vocabulary: Reset Freq "Once" (was
Inception), "Start Date" header (was Open), and a new optional "Inception"
column in the example/template xlsx + Instructions. Regenerate
overview.html/png and the bundled example-portfolio.xlsx / template.xlsx
(and the app/assets copies).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/assets/example-portfolio.xlsx
+++ b/app/assets/example-portfolio.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X13"/>
+  <dimension ref="A1:Y13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -468,6 +468,7 @@
     <col width="15" customWidth="1" min="22" max="22"/>
     <col width="15" customWidth="1" min="23" max="23"/>
     <col width="15" customWidth="1" min="24" max="24"/>
+    <col width="15" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -587,7 +588,7 @@
       </c>
       <c r="U3" s="1" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Start Date</t>
         </is>
       </c>
       <c r="V3" s="1" t="inlineStr">
@@ -603,6 +604,11 @@
       <c r="X3" s="1" t="inlineStr">
         <is>
           <t>RUT_Strike</t>
+        </is>
+      </c>
+      <c r="Y3" s="1" t="inlineStr">
+        <is>
+          <t>Inception</t>
         </is>
       </c>
     </row>
@@ -687,6 +693,7 @@
       </c>
       <c r="W4" s="5" t="n"/>
       <c r="X4" s="5" t="n"/>
+      <c r="Y4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -758,7 +765,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Inception</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="U5" s="4" t="n">
@@ -769,6 +776,7 @@
       </c>
       <c r="W5" s="5" t="n"/>
       <c r="X5" s="5" t="n"/>
+      <c r="Y5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -840,7 +848,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Inception</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="U6" s="4" t="n">
@@ -851,6 +859,7 @@
       </c>
       <c r="W6" s="5" t="n"/>
       <c r="X6" s="5" t="n"/>
+      <c r="Y6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -922,7 +931,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Inception</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="U7" s="4" t="n">
@@ -933,6 +942,7 @@
       </c>
       <c r="W7" s="5" t="n"/>
       <c r="X7" s="5" t="n"/>
+      <c r="Y7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1004,7 +1014,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>Inception</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="U8" s="4" t="n">
@@ -1015,6 +1025,7 @@
       </c>
       <c r="W8" s="5" t="n"/>
       <c r="X8" s="5" t="n"/>
+      <c r="Y8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1101,6 +1112,7 @@
       <c r="X9" s="5" t="n">
         <v>2719</v>
       </c>
+      <c r="Y9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1172,7 +1184,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>Inception</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="U10" s="4" t="n">
@@ -1183,6 +1195,7 @@
       </c>
       <c r="W10" s="5" t="n"/>
       <c r="X10" s="5" t="n"/>
+      <c r="Y10" s="4" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1254,7 +1267,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>Inception</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="U11" s="4" t="n">
@@ -1265,6 +1278,7 @@
       </c>
       <c r="W11" s="5" t="n"/>
       <c r="X11" s="5" t="n"/>
+      <c r="Y11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1336,7 +1350,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>Inception</t>
+          <t>Once</t>
         </is>
       </c>
       <c r="U12" s="4" t="n">
@@ -1347,6 +1361,7 @@
       </c>
       <c r="W12" s="5" t="n"/>
       <c r="X12" s="5" t="n"/>
+      <c r="Y12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -1385,6 +1400,7 @@
       <c r="V13" s="9" t="n"/>
       <c r="W13" s="10" t="n"/>
       <c r="X13" s="10" t="n"/>
+      <c r="Y13" s="9" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sample portfolio: $10K positions instead of $100K (v1.6.5)
Scale every $000 column (Initial, Realized, Proj Value, Proj $ Gain) and
the TOTAL row in the bundled + docs example portfolios by 0.1, so each
sample holding shows a $10K investment. Ratios/prices (cap, participation,
floor, strike, %) unchanged. Proj Value/Proj $ Gain are recomputed on
import; scaling them only keeps the file self-consistent when opened in Excel.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/assets/example-portfolio.xlsx
+++ b/app/assets/example-portfolio.xlsx
@@ -639,16 +639,16 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>112.25</v>
+        <v>11.225</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>12.25</v>
+        <v>1.225</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>0.1225</v>
@@ -722,16 +722,16 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>93</v>
+        <v>9.3</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>-7.000000000000001</v>
+        <v>-0.7</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>-0.07000000000000001</v>
@@ -805,16 +805,16 @@
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>130.6</v>
+        <v>13.06</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>30.6</v>
+        <v>3.06</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>0.306</v>
@@ -888,16 +888,16 @@
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>136.9</v>
+        <v>13.69</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>36.9</v>
+        <v>3.69</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>0.369</v>
@@ -971,16 +971,16 @@
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>65</v>
+        <v>6.5</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>-35</v>
+        <v>-3.5</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>-0.35</v>
@@ -1054,16 +1054,16 @@
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>1.1</v>
+        <v>0.11</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>102.2163125</v>
+        <v>10.22163125</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>1.1163125</v>
+        <v>0.11163125</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>0.01104166666666667</v>
@@ -1141,13 +1141,13 @@
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="I10" s="2" t="n">
         <v>0</v>
@@ -1224,16 +1224,16 @@
         </is>
       </c>
       <c r="F11" s="2" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>112</v>
+        <v>11.2</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>12</v>
+        <v>1.2</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>0.12</v>
@@ -1307,16 +1307,16 @@
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>90</v>
+        <v>9</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>-10</v>
+        <v>-1</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>-0.1</v>
@@ -1374,16 +1374,16 @@
       <c r="D13" s="6" t="n"/>
       <c r="E13" s="6" t="n"/>
       <c r="F13" s="7" t="n">
-        <v>900</v>
+        <v>90</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>1.1</v>
+        <v>0.11</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>941.9663125</v>
+        <v>94.19663125</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>40.86631249999999</v>
+        <v>4.08663125</v>
       </c>
       <c r="J13" s="8" t="n"/>
       <c r="K13" s="8" t="n"/>

</xml_diff>

<commit_message>
Sample portfolio: $10K positions instead of $100K (v1.6.5) (#13)
Scale every $000 column (Initial, Realized, Proj Value, Proj $ Gain) and
the TOTAL row in the bundled + docs example portfolios by 0.1, so each
sample holding shows a $10K investment. Ratios/prices (cap, participation,
floor, strike, %) unchanged. Proj Value/Proj $ Gain are recomputed on
import; scaling them only keeps the file self-consistent when opened in Excel.

Co-authored-by: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/assets/example-portfolio.xlsx
+++ b/app/assets/example-portfolio.xlsx
@@ -639,16 +639,16 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>112.25</v>
+        <v>11.225</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>12.25</v>
+        <v>1.225</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>0.1225</v>
@@ -722,16 +722,16 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>93</v>
+        <v>9.3</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>-7.000000000000001</v>
+        <v>-0.7</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>-0.07000000000000001</v>
@@ -805,16 +805,16 @@
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>130.6</v>
+        <v>13.06</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>30.6</v>
+        <v>3.06</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>0.306</v>
@@ -888,16 +888,16 @@
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>136.9</v>
+        <v>13.69</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>36.9</v>
+        <v>3.69</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>0.369</v>
@@ -971,16 +971,16 @@
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>65</v>
+        <v>6.5</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>-35</v>
+        <v>-3.5</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>-0.35</v>
@@ -1054,16 +1054,16 @@
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>1.1</v>
+        <v>0.11</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>102.2163125</v>
+        <v>10.22163125</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>1.1163125</v>
+        <v>0.11163125</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>0.01104166666666667</v>
@@ -1141,13 +1141,13 @@
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="I10" s="2" t="n">
         <v>0</v>
@@ -1224,16 +1224,16 @@
         </is>
       </c>
       <c r="F11" s="2" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>112</v>
+        <v>11.2</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>12</v>
+        <v>1.2</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>0.12</v>
@@ -1307,16 +1307,16 @@
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>90</v>
+        <v>9</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>-10</v>
+        <v>-1</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>-0.1</v>
@@ -1374,16 +1374,16 @@
       <c r="D13" s="6" t="n"/>
       <c r="E13" s="6" t="n"/>
       <c r="F13" s="7" t="n">
-        <v>900</v>
+        <v>90</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>1.1</v>
+        <v>0.11</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>941.9663125</v>
+        <v>94.19663125</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>40.86631249999999</v>
+        <v>4.08663125</v>
       </c>
       <c r="J13" s="8" t="n"/>
       <c r="K13" s="8" t="n"/>

</xml_diff>

<commit_message>
Fix CI + docs for the $10K sample; regenerate from gen_overview.py (v1.6.6)
The v1.6.5 sample change ($100K→$10K) was hand-edited into the xlsx binaries,
which broke three tests that hard-code the old dollar figures and left the docs
still showing $100K.

- Make gen_overview.py the single source: add PRINCIPAL=10.0, scale the note's
  realized coupon 1.10→0.11 for a uniform 1/10 sample, and regenerate all four
  xlsx files (data/ + app/assets/) plus overview.html.
- Update the three tests to the $10K figures (Proj Value, realized, totals).
- Update README (heading, intro, Proj Value column, total) and regenerate
  docs/overview.png + docs/screenshots/{hero,drilldown,phone-cards}.png.

flutter test --exclude-tags golden: 247 pass. Coverage gate holds (core 100%,
data 96.79%). Goldens regenerated and copied to docs/screenshots.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/assets/example-portfolio.xlsx
+++ b/app/assets/example-portfolio.xlsx
@@ -728,10 +728,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>9.3</v>
+        <v>9.299999999999999</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>-0.7</v>
+        <v>-0.7000000000000001</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>-0.07000000000000001</v>

</xml_diff>

<commit_message>
Fix CI + docs for the $10K sample; regenerate from gen_overview.py (v1.6.6) (#14)
The v1.6.5 sample change ($100K→$10K) was hand-edited into the xlsx binaries,
which broke three tests that hard-code the old dollar figures and left the docs
still showing $100K.

- Make gen_overview.py the single source: add PRINCIPAL=10.0, scale the note's
  realized coupon 1.10→0.11 for a uniform 1/10 sample, and regenerate all four
  xlsx files (data/ + app/assets/) plus overview.html.
- Update the three tests to the $10K figures (Proj Value, realized, totals).
- Update README (heading, intro, Proj Value column, total) and regenerate
  docs/overview.png + docs/screenshots/{hero,drilldown,phone-cards}.png.

flutter test --exclude-tags golden: 247 pass. Coverage gate holds (core 100%,
data 96.79%). Goldens regenerated and copied to docs/screenshots.

Co-authored-by: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/assets/example-portfolio.xlsx
+++ b/app/assets/example-portfolio.xlsx
@@ -728,10 +728,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>9.3</v>
+        <v>9.299999999999999</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>-0.7</v>
+        <v>-0.7000000000000001</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>-0.07000000000000001</v>

</xml_diff>